<commit_message>
fixed : using Quantlib
</commit_message>
<xml_diff>
--- a/PricingSheet_template.xlsx
+++ b/PricingSheet_template.xlsx
@@ -1181,7 +1181,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X100"/>
+  <dimension ref="A1:W100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" bestFit="1" customWidth="1" min="3" max="3"/>
@@ -1196,115 +1196,110 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>hist_flag</t>
+          <t>risk_flag</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>risk_flag</t>
+          <t>remarks</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>remarks</t>
+          <t>notional</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>notional</t>
+          <t>delta</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
+          <t>adj_notional</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>start</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>tenor</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>end</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>fix rate</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>fix freq</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>fix dcf</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>index</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>float freq</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>float dcf</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>roll conv</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>target fixrate</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>spred</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>fly</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>pay/rec</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>PV</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
           <t>delta</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>adj_notional</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>start</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>tenor</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>end</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>fix rate</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>fix freq</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>fix dcf</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>index</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>float freq</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>float dcf</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>roll conv</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>target fixrate</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>spred</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr">
-        <is>
-          <t>fly</t>
-        </is>
-      </c>
-      <c r="U1" t="inlineStr">
-        <is>
-          <t>pay/rec</t>
-        </is>
-      </c>
-      <c r="V1" t="inlineStr">
-        <is>
-          <t>PV</t>
-        </is>
-      </c>
       <c r="W1" t="inlineStr">
-        <is>
-          <t>delta</t>
-        </is>
-      </c>
-      <c r="X1" t="inlineStr">
         <is>
           <t>delta(annuity)</t>
         </is>
@@ -1314,67 +1309,67 @@
       <c r="A2" t="n">
         <v>1</v>
       </c>
-      <c r="C2" t="n">
+      <c r="B2" t="n">
         <v>0</v>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>test</t>
         </is>
       </c>
-      <c r="E2" t="n">
+      <c r="D2" t="n">
         <v>1000000000</v>
       </c>
-      <c r="H2" s="2" t="n">
+      <c r="G2" s="2" t="n">
         <v>46233</v>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>2y</t>
         </is>
       </c>
-      <c r="J2" s="2" t="n">
+      <c r="I2" s="2" t="n">
         <v>46965</v>
       </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>PA</t>
+        </is>
+      </c>
       <c r="L2" t="inlineStr">
         <is>
+          <t>act/365fixed</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>JSCC</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
           <t>PA</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="O2" t="inlineStr">
         <is>
           <t>act/365fixed</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>JSCC</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>PA</t>
-        </is>
-      </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>act/365fixed</t>
-        </is>
-      </c>
-      <c r="Q2" t="inlineStr">
-        <is>
           <t>STD</t>
         </is>
       </c>
-      <c r="R2" t="n">
+      <c r="Q2" t="n">
         <v>1.62075225387002</v>
       </c>
-      <c r="U2" t="inlineStr">
+      <c r="T2" t="inlineStr">
         <is>
           <t>PAY</t>
         </is>
       </c>
-      <c r="V2" t="n">
+      <c r="U2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1382,67 +1377,67 @@
       <c r="A3" t="n">
         <v>1</v>
       </c>
-      <c r="C3" t="n">
+      <c r="B3" t="n">
         <v>0</v>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>test</t>
         </is>
       </c>
-      <c r="E3" t="n">
+      <c r="D3" t="n">
         <v>1000000000</v>
       </c>
-      <c r="H3" s="2" t="n">
+      <c r="G3" s="2" t="n">
         <v>46233</v>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>5y</t>
         </is>
       </c>
-      <c r="J3" s="2" t="n">
+      <c r="I3" s="2" t="n">
         <v>48059</v>
       </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>PA</t>
+        </is>
+      </c>
       <c r="L3" t="inlineStr">
         <is>
+          <t>act/365fixed</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>JSCC</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
           <t>PA</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="O3" t="inlineStr">
         <is>
           <t>act/365fixed</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>JSCC</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>PA</t>
-        </is>
-      </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>act/365fixed</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
           <t>STD</t>
         </is>
       </c>
-      <c r="R3" t="n">
+      <c r="Q3" t="n">
         <v>2.085701110110807</v>
       </c>
-      <c r="U3" t="inlineStr">
+      <c r="T3" t="inlineStr">
         <is>
           <t>PAY</t>
         </is>
       </c>
-      <c r="V3" t="n">
+      <c r="U3" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1450,70 +1445,165 @@
       <c r="A4" t="n">
         <v>1</v>
       </c>
-      <c r="C4" t="n">
+      <c r="B4" t="n">
         <v>0</v>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>test</t>
         </is>
       </c>
-      <c r="E4" t="n">
+      <c r="D4" t="n">
         <v>1000000000</v>
       </c>
-      <c r="H4" s="2" t="n">
+      <c r="G4" s="2" t="n">
         <v>46233</v>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>10y</t>
         </is>
       </c>
-      <c r="J4" s="2" t="n">
+      <c r="I4" s="2" t="n">
         <v>49886</v>
       </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>PA</t>
+        </is>
+      </c>
       <c r="L4" t="inlineStr">
         <is>
+          <t>act/365fixed</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>JSCC</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
           <t>PA</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="O4" t="inlineStr">
         <is>
           <t>act/365fixed</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>JSCC</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>PA</t>
-        </is>
-      </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>act/365fixed</t>
-        </is>
-      </c>
-      <c r="Q4" t="inlineStr">
-        <is>
           <t>STD</t>
         </is>
       </c>
-      <c r="R4" t="n">
+      <c r="Q4" t="n">
         <v>2.64428108086317</v>
       </c>
-      <c r="U4" t="inlineStr">
+      <c r="T4" t="inlineStr">
         <is>
           <t>PAY</t>
         </is>
       </c>
-      <c r="V4" t="n">
+      <c r="U4" t="n">
         <v>0</v>
       </c>
     </row>
+    <row r="5"/>
+    <row r="6"/>
+    <row r="7"/>
+    <row r="8"/>
+    <row r="9"/>
+    <row r="10"/>
+    <row r="11"/>
+    <row r="12"/>
+    <row r="13"/>
+    <row r="14"/>
+    <row r="15"/>
+    <row r="16"/>
+    <row r="17"/>
+    <row r="18"/>
+    <row r="19"/>
+    <row r="20"/>
+    <row r="21"/>
+    <row r="22"/>
+    <row r="23"/>
+    <row r="24"/>
+    <row r="25"/>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
+    <row r="40"/>
+    <row r="41"/>
+    <row r="42"/>
+    <row r="43"/>
+    <row r="44"/>
+    <row r="45"/>
+    <row r="46"/>
+    <row r="47"/>
+    <row r="48"/>
+    <row r="49"/>
+    <row r="50"/>
+    <row r="51"/>
+    <row r="52"/>
+    <row r="53"/>
+    <row r="54"/>
+    <row r="55"/>
+    <row r="56"/>
+    <row r="57"/>
+    <row r="58"/>
+    <row r="59"/>
+    <row r="60"/>
+    <row r="61"/>
+    <row r="62"/>
+    <row r="63"/>
+    <row r="64"/>
+    <row r="65"/>
+    <row r="66"/>
+    <row r="67"/>
+    <row r="68"/>
+    <row r="69"/>
+    <row r="70"/>
+    <row r="71"/>
+    <row r="72"/>
+    <row r="73"/>
+    <row r="74"/>
+    <row r="75"/>
+    <row r="76"/>
+    <row r="77"/>
+    <row r="78"/>
+    <row r="79"/>
+    <row r="80"/>
+    <row r="81"/>
+    <row r="82"/>
+    <row r="83"/>
+    <row r="84"/>
+    <row r="85"/>
+    <row r="86"/>
+    <row r="87"/>
+    <row r="88"/>
+    <row r="89"/>
+    <row r="90"/>
+    <row r="91"/>
+    <row r="92"/>
+    <row r="93"/>
+    <row r="94"/>
+    <row r="95"/>
+    <row r="96"/>
+    <row r="97"/>
+    <row r="98"/>
+    <row r="99"/>
     <row r="100">
       <c r="A100" t="n">
         <v>0</v>
@@ -1521,25 +1611,25 @@
     </row>
   </sheetData>
   <dataValidations count="7">
-    <dataValidation sqref="J2:J200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="L2:L200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"PA,SA,QA,1m"</formula1>
+    </dataValidation>
+    <dataValidation sqref="O2:O200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"PA,SA,QA,1m"</formula1>
     </dataValidation>
     <dataValidation sqref="M2:M200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>"PA,SA,QA,1m"</formula1>
+      <formula1>"act/365fixed,30/360"</formula1>
     </dataValidation>
-    <dataValidation sqref="K2:K200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="P2:P200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"act/365fixed,30/360"</formula1>
     </dataValidation>
     <dataValidation sqref="N2:N200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>"act/365fixed,30/360"</formula1>
-    </dataValidation>
-    <dataValidation sqref="L2:L200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"JSCC"</formula1>
     </dataValidation>
-    <dataValidation sqref="O2:O200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="Q2:Q200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"STD,EOM,IMM"</formula1>
     </dataValidation>
-    <dataValidation sqref="S2:S200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="U2:U200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"PAY,REC"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1553,7 +1643,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BE278"/>
+  <dimension ref="A1:H278"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">

</xml_diff>

<commit_message>
fixed : maked UDF in VBA
</commit_message>
<xml_diff>
--- a/PricingSheet_template.xlsx
+++ b/PricingSheet_template.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Historical" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="191028" fullCalcOnLoad="1"/>
+  <calcPr calcId="191028" calcMode="manual" fullCalcOnLoad="0"/>
 </workbook>
 </file>
 
@@ -1509,101 +1509,6 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5"/>
-    <row r="6"/>
-    <row r="7"/>
-    <row r="8"/>
-    <row r="9"/>
-    <row r="10"/>
-    <row r="11"/>
-    <row r="12"/>
-    <row r="13"/>
-    <row r="14"/>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
-    <row r="60"/>
-    <row r="61"/>
-    <row r="62"/>
-    <row r="63"/>
-    <row r="64"/>
-    <row r="65"/>
-    <row r="66"/>
-    <row r="67"/>
-    <row r="68"/>
-    <row r="69"/>
-    <row r="70"/>
-    <row r="71"/>
-    <row r="72"/>
-    <row r="73"/>
-    <row r="74"/>
-    <row r="75"/>
-    <row r="76"/>
-    <row r="77"/>
-    <row r="78"/>
-    <row r="79"/>
-    <row r="80"/>
-    <row r="81"/>
-    <row r="82"/>
-    <row r="83"/>
-    <row r="84"/>
-    <row r="85"/>
-    <row r="86"/>
-    <row r="87"/>
-    <row r="88"/>
-    <row r="89"/>
-    <row r="90"/>
-    <row r="91"/>
-    <row r="92"/>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
     <row r="100">
       <c r="A100" t="n">
         <v>0</v>

</xml_diff>